<commit_message>
Se estuvo llenado las registros del muestreo faltante
</commit_message>
<xml_diff>
--- a/servicios.xlsx
+++ b/servicios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/120f6d501c463b80/Escritorio/leo/Doo/Barberia proyecto/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="171" documentId="11_AD4D2F04E46CFB4ACB3E20F07552DBC0683EDF10" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A14045C-B962-4270-AF5D-D2C0E94459A9}"/>
+  <xr:revisionPtr revIDLastSave="184" documentId="11_AD4D2F04E46CFB4ACB3E20F07552DBC0683EDF10" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D26BAD2-83FA-4C3F-8849-52F03C0B807C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="57">
   <si>
     <t>Servicio</t>
   </si>
@@ -198,6 +198,15 @@
   </si>
   <si>
     <t>Sacar del catalogo un servicio</t>
+  </si>
+  <si>
+    <t>Definir las políticas de la barbería</t>
+  </si>
+  <si>
+    <t>Modificar las políticas</t>
+  </si>
+  <si>
+    <t>Ver la regla definida</t>
   </si>
 </sst>
 </file>
@@ -300,7 +309,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -317,8 +326,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -615,6 +622,7 @@
     <col min="9" max="9" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="32.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="17.85546875" customWidth="1"/>
+    <col min="14" max="14" width="30.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:18" x14ac:dyDescent="0.25">
@@ -706,8 +714,12 @@
       <c r="L4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
+      <c r="N4" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>4</v>
+      </c>
       <c r="Q4" s="3"/>
       <c r="R4" s="3"/>
     </row>
@@ -730,8 +742,12 @@
       <c r="L5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="N5" s="4"/>
-      <c r="O5" s="4"/>
+      <c r="N5" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>4</v>
+      </c>
       <c r="Q5" s="4"/>
       <c r="R5" s="4"/>
     </row>
@@ -754,8 +770,12 @@
       <c r="L6" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="N6" s="3"/>
-      <c r="O6" s="4"/>
+      <c r="N6" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>4</v>
+      </c>
       <c r="Q6" s="3"/>
       <c r="R6" s="4"/>
     </row>
@@ -778,8 +798,8 @@
       <c r="L7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="N7" s="3"/>
-      <c r="O7" s="3"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
       <c r="Q7" s="3"/>
       <c r="R7" s="3"/>
     </row>
@@ -904,7 +924,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B25" s="4" t="s">
         <v>39</v>
       </c>
@@ -951,7 +971,7 @@
       </c>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="E29" s="8" t="s">
+      <c r="E29" s="3" t="s">
         <v>51</v>
       </c>
       <c r="F29" s="3" t="s">
@@ -959,7 +979,7 @@
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="E30" s="8" t="s">
+      <c r="E30" s="3" t="s">
         <v>52</v>
       </c>
       <c r="F30" s="3" t="s">
@@ -967,36 +987,20 @@
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="E31" s="8" t="s">
+      <c r="E31" s="3" t="s">
         <v>53</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="E32" s="9"/>
-      <c r="F32" s="10"/>
-    </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="E33" s="9"/>
-      <c r="F33" s="10"/>
-    </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="E34" s="9"/>
-      <c r="F34" s="10"/>
-    </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="E35" s="9"/>
-      <c r="F35" s="10"/>
-    </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B36" s="5" t="s">
         <v>30</v>
       </c>
       <c r="C36" s="5"/>
     </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B37" s="1" t="s">
         <v>1</v>
       </c>
@@ -1004,7 +1008,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B38" s="3" t="s">
         <v>44</v>
       </c>
@@ -1012,25 +1016,25 @@
         <v>45</v>
       </c>
     </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B39" s="4"/>
       <c r="C39" s="3"/>
     </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B40" s="3"/>
       <c r="C40" s="4"/>
     </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
     </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B46" s="5" t="s">
         <v>31</v>
       </c>
       <c r="C46" s="5"/>
     </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B47" s="1" t="s">
         <v>1</v>
       </c>
@@ -1038,7 +1042,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B48" s="3" t="s">
         <v>41</v>
       </c>

</xml_diff>

<commit_message>
Se definieron los servicios para el modelo de dominio
</commit_message>
<xml_diff>
--- a/servicios.xlsx
+++ b/servicios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/120f6d501c463b80/Escritorio/leo/Doo/Barberia proyecto/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="184" documentId="11_AD4D2F04E46CFB4ACB3E20F07552DBC0683EDF10" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D26BAD2-83FA-4C3F-8849-52F03C0B807C}"/>
+  <xr:revisionPtr revIDLastSave="303" documentId="11_AD4D2F04E46CFB4ACB3E20F07552DBC0683EDF10" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D794696-95F7-477C-9FBB-84085CBA736E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="80">
   <si>
     <t>Servicio</t>
   </si>
@@ -47,54 +47,24 @@
     <t>Actor</t>
   </si>
   <si>
-    <t xml:space="preserve">Ofrecer un servicio nuevo </t>
-  </si>
-  <si>
     <t>Dueño</t>
   </si>
   <si>
-    <t>Ajustar las propiedades de un servicio</t>
-  </si>
-  <si>
-    <t>Ver servicios disponibles</t>
-  </si>
-  <si>
     <t>Dueño, Barbero, Cliente</t>
   </si>
   <si>
-    <t>Retirar un servicio</t>
-  </si>
-  <si>
     <t>PrefijoCelular</t>
   </si>
   <si>
     <t>Barbero, Cliente</t>
   </si>
   <si>
-    <t>Lo mismo que con prefijo, se tiene definido o se va a definir</t>
-  </si>
-  <si>
     <t>Estado</t>
   </si>
   <si>
-    <t>Seleccionar estado</t>
-  </si>
-  <si>
-    <t>Creo que seleccionar en prefijo y en estado no corresponden</t>
-  </si>
-  <si>
-    <t>Ver estados</t>
-  </si>
-  <si>
-    <t>Editar descripcion de Estado</t>
-  </si>
-  <si>
     <t>TipoMulta</t>
   </si>
   <si>
-    <t>Lo mismo</t>
-  </si>
-  <si>
     <t>Ver tipos de multa</t>
   </si>
   <si>
@@ -146,18 +116,12 @@
     <t>Definir horario de barberia</t>
   </si>
   <si>
-    <t>Ver horario de barberia</t>
-  </si>
-  <si>
     <t>Desactivar horario de barberia</t>
   </si>
   <si>
     <t>Definir mi horario de trabajo</t>
   </si>
   <si>
-    <t>Ver horario horario de barbero</t>
-  </si>
-  <si>
     <t>Desactivar horario de trabajo</t>
   </si>
   <si>
@@ -207,6 +171,111 @@
   </si>
   <si>
     <t>Ver la regla definida</t>
+  </si>
+  <si>
+    <t>Editar tiempos de anticipacion de citas</t>
+  </si>
+  <si>
+    <t>Ver número del barbero</t>
+  </si>
+  <si>
+    <t>Dejar de trabajar en la barberia</t>
+  </si>
+  <si>
+    <t>Editar mi contacto</t>
+  </si>
+  <si>
+    <t>Ver número del cliente</t>
+  </si>
+  <si>
+    <t>Ver mis multas multas sin pagar</t>
+  </si>
+  <si>
+    <t>Estoy vetado</t>
+  </si>
+  <si>
+    <t>Registrar barbero a la barberia</t>
+  </si>
+  <si>
+    <t>Registrar cliente a la barberia</t>
+  </si>
+  <si>
+    <t>Ajustar los datos del servicio</t>
+  </si>
+  <si>
+    <t>Ofrecer un servicio nuevo a la barberia</t>
+  </si>
+  <si>
+    <t>Retirar un servicio de la barberia</t>
+  </si>
+  <si>
+    <t>Ver servicios disponibles de la barberia</t>
+  </si>
+  <si>
+    <t>Ver prefijos de celular</t>
+  </si>
+  <si>
+    <t>Definir tipo de multa para el cliente</t>
+  </si>
+  <si>
+    <t>Ver estados creados</t>
+  </si>
+  <si>
+    <t>Editar descripcion del estado de las citas</t>
+  </si>
+  <si>
+    <t>Editar nombre del estado de las citas</t>
+  </si>
+  <si>
+    <t>Definir tipo de estado de las citas</t>
+  </si>
+  <si>
+    <t>Ver cuantos descuentos tengo para mis futuras citas</t>
+  </si>
+  <si>
+    <t>Ver dia de la semana</t>
+  </si>
+  <si>
+    <t>Ver los dias de las semanas</t>
+  </si>
+  <si>
+    <t>Ver horarios de la barberia</t>
+  </si>
+  <si>
+    <t>Ver mis horarios definidos</t>
+  </si>
+  <si>
+    <t>Ver horarios de trabajo de un barbero</t>
+  </si>
+  <si>
+    <t>Ver citas agendas</t>
+  </si>
+  <si>
+    <t>Cambiar a estado de retraso</t>
+  </si>
+  <si>
+    <t>Cambiar a estado de finalizada</t>
+  </si>
+  <si>
+    <t>Cambiar a estado de inasistencia por el cliente</t>
+  </si>
+  <si>
+    <t>Cambiar a estado de inasistencia por el barbero</t>
+  </si>
+  <si>
+    <t>O sera mejor el sistema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generar multa </t>
+  </si>
+  <si>
+    <t>Ver todas mis multas</t>
+  </si>
+  <si>
+    <t>La multa se pago</t>
+  </si>
+  <si>
+    <t>O sera mejor cliente</t>
   </si>
 </sst>
 </file>
@@ -309,7 +378,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -326,7 +395,18 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -611,18 +691,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:R61"/>
+  <dimension ref="B2:R66"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.42578125" customWidth="1"/>
     <col min="5" max="5" width="45.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.42578125" customWidth="1"/>
-    <col min="8" max="8" width="54.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="35.42578125" customWidth="1"/>
     <col min="9" max="9" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="32.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="17.85546875" customWidth="1"/>
     <col min="14" max="14" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:18" x14ac:dyDescent="0.25">
@@ -631,23 +712,23 @@
       </c>
       <c r="C2" s="5"/>
       <c r="E2" s="5" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F2" s="5"/>
       <c r="H2" s="5" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="I2" s="5"/>
       <c r="K2" s="6" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="L2" s="7"/>
       <c r="N2" s="6" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="O2" s="7"/>
       <c r="Q2" s="6" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="R2" s="7"/>
     </row>
@@ -689,136 +770,143 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B4" s="3" t="s">
+    <row r="4" spans="2:18" ht="30" x14ac:dyDescent="0.25">
+      <c r="B4" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="E4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="R4" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="2:18" ht="30" x14ac:dyDescent="0.25">
+      <c r="B5" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="L5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="I4" s="3" t="s">
+      <c r="N5" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q5" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="R5" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="2:18" ht="30" x14ac:dyDescent="0.25">
+      <c r="B6" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="N4" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="O4" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
-    </row>
-    <row r="5" spans="2:18" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="N5" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="O5" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="Q5" s="4"/>
-      <c r="R5" s="4"/>
-    </row>
-    <row r="6" spans="2:18" ht="30" x14ac:dyDescent="0.25">
-      <c r="B6" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>7</v>
-      </c>
       <c r="H6" s="3" t="s">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="Q6" s="3"/>
-      <c r="R6" s="4"/>
+        <v>12</v>
+      </c>
+      <c r="Q6" s="11"/>
+      <c r="R6" s="12"/>
     </row>
     <row r="7" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
-        <v>8</v>
+        <v>56</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>16</v>
+        <v>61</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="N7" s="8"/>
-      <c r="O7" s="8"/>
-      <c r="Q7" s="3"/>
-      <c r="R7" s="3"/>
-    </row>
-    <row r="9" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="H9" t="s">
-        <v>14</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="Q7" s="11"/>
+      <c r="R7" s="11"/>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B12" s="5" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="C12" s="5"/>
       <c r="E12" s="5" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F12" s="5"/>
       <c r="H12" s="5" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="I12" s="5"/>
     </row>
@@ -844,285 +932,409 @@
     </row>
     <row r="14" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="C14" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="2:18" ht="30" x14ac:dyDescent="0.25">
+      <c r="B15" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-    </row>
-    <row r="15" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B15" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E15" s="4"/>
-      <c r="F15" s="3"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="3"/>
+      <c r="E15" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="16" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="E17" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="E18" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="I18" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="H19" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="I19" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+    </row>
+    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="H23" s="9"/>
+      <c r="I23" s="9"/>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B25" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" s="5"/>
+      <c r="E25" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F25" s="5"/>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B26" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B27" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B28" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B29" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B30" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E30" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E16" s="3"/>
-      <c r="F16" s="4"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="4"/>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-    </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B22" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C22" s="5"/>
-      <c r="E22" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F22" s="5"/>
-    </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B23" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B24" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B25" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B26" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="E27" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="E28" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="E29" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="E30" s="3" t="s">
-        <v>52</v>
-      </c>
       <c r="F30" s="3" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.25">
       <c r="E31" s="3" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B36" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="E32" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E33" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E34" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B39" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C39" s="5"/>
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B40" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B41" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B42" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B43" s="3"/>
+      <c r="C43" s="4"/>
+    </row>
+    <row r="44" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B44" s="3"/>
+      <c r="C44" s="3"/>
+    </row>
+    <row r="49" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B49" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C49" s="5"/>
+    </row>
+    <row r="50" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B50" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B51" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="52" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B52" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C36" s="5"/>
-    </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B37" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B38" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B39" s="4"/>
-      <c r="C39" s="3"/>
-    </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B40" s="3"/>
-      <c r="C40" s="4"/>
-    </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B41" s="3"/>
-      <c r="C41" s="3"/>
-    </row>
-    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B46" s="5" t="s">
+      <c r="C52" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C46" s="5"/>
-    </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B47" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B48" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="49" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B49" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="50" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B50" s="3"/>
-      <c r="C50" s="4"/>
-    </row>
-    <row r="51" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B51" s="3"/>
-      <c r="C51" s="3"/>
-    </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B56" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C56" s="5"/>
-      <c r="E56" s="5" t="s">
+    </row>
+    <row r="53" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B53" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C53" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F56" s="5"/>
+    </row>
+    <row r="54" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B54" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="55" spans="2:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="B55" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="C55" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="56" spans="2:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="B56" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D56" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="57" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B57" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F57" s="2" t="s">
-        <v>2</v>
-      </c>
+      <c r="B57" s="13"/>
+      <c r="C57" s="9"/>
     </row>
     <row r="58" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B58" s="3"/>
-      <c r="C58" s="3"/>
-      <c r="E58" s="3"/>
-      <c r="F58" s="3"/>
-    </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B59" s="4"/>
-      <c r="C59" s="3"/>
-      <c r="E59" s="4"/>
-      <c r="F59" s="3"/>
-    </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B60" s="3"/>
-      <c r="C60" s="4"/>
-      <c r="E60" s="3"/>
-      <c r="F60" s="4"/>
+      <c r="B58" s="13"/>
+      <c r="C58" s="9"/>
     </row>
     <row r="61" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B61" s="3"/>
-      <c r="C61" s="3"/>
-      <c r="E61" s="3"/>
-      <c r="F61" s="3"/>
+      <c r="B61" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C61" s="5"/>
+      <c r="E61" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F61" s="5"/>
+    </row>
+    <row r="62" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B62" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B63" s="3"/>
+      <c r="C63" s="3"/>
+      <c r="E63" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F63" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="64" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B64" s="4"/>
+      <c r="C64" s="3"/>
+      <c r="E64" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F64" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="65" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B65" s="3"/>
+      <c r="C65" s="4"/>
+      <c r="E65" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F65" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G65" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="66" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B66" s="3"/>
+      <c r="C66" s="3"/>
+      <c r="E66" s="3"/>
+      <c r="F66" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B56:C56"/>
-    <mergeCell ref="E56:F56"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="E61:F61"/>
     <mergeCell ref="Q2:R2"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="B39:C39"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>

</xml_diff>

<commit_message>
Se hiceiron los cambios al modelo de dominio, al muestreo y a los eventos
</commit_message>
<xml_diff>
--- a/servicios.xlsx
+++ b/servicios.xlsx
@@ -5,22 +5,35 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jesus\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Desktop\DOO\DOO\Barberia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85C37906-837E-4637-AA86-A88883909B3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AB46960-CA2B-4571-925B-D430D14FB839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Responsablidades" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="80">
   <si>
     <t>Servicio</t>
   </si>
@@ -76,9 +89,6 @@
     <t>Dueño, Barbero</t>
   </si>
   <si>
-    <t>Ajustar el nombre y la descripcion de un servicio</t>
-  </si>
-  <si>
     <t>Modificar las políticas</t>
   </si>
   <si>
@@ -196,18 +206,12 @@
     <t>Pedir cita</t>
   </si>
   <si>
-    <t>Bloquear un espacio de la agenda</t>
-  </si>
-  <si>
     <t>Reprogramar la cita</t>
   </si>
   <si>
     <t>Cancelar la cita por decisión del cliente</t>
   </si>
   <si>
-    <t>Consultar los bloqueos de una agenda</t>
-  </si>
-  <si>
     <t>Cancelar la cita por decisión del barbero</t>
   </si>
   <si>
@@ -247,10 +251,28 @@
     <t>Editar descripcion del estado</t>
   </si>
   <si>
-    <t>Cancelar un bloqueo de la agenda</t>
-  </si>
-  <si>
     <t>Ver precio de cada servicio</t>
+  </si>
+  <si>
+    <t>Definir un bloque de no disponible</t>
+  </si>
+  <si>
+    <t>Borrar un bloqueo</t>
+  </si>
+  <si>
+    <t>Ver bloqueos en un rango de fechas</t>
+  </si>
+  <si>
+    <t>Ver bloqueos de una fecha</t>
+  </si>
+  <si>
+    <t>Ajustar el nombre de un servicio</t>
+  </si>
+  <si>
+    <t>Ajustar la descripcion de un servicio</t>
+  </si>
+  <si>
+    <t>Ver descripción de un estado</t>
   </si>
 </sst>
 </file>
@@ -276,6 +298,7 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -351,7 +374,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -363,12 +386,15 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -649,48 +675,49 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:R59"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:R60"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="41.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" customWidth="1"/>
-    <col min="5" max="5" width="42.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.42578125" customWidth="1"/>
-    <col min="8" max="8" width="35.42578125" customWidth="1"/>
-    <col min="9" max="9" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="32.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.85546875" customWidth="1"/>
-    <col min="14" max="14" width="30.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="41.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.44140625" customWidth="1"/>
+    <col min="5" max="5" width="42.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.44140625" customWidth="1"/>
+    <col min="8" max="8" width="35.44140625" customWidth="1"/>
+    <col min="9" max="9" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="32.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.88671875" customWidth="1"/>
+    <col min="14" max="14" width="30.5546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.44140625" customWidth="1"/>
+    <col min="17" max="17" width="19.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B2" s="7" t="s">
+    <row r="2" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="B2" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="E2" s="7" t="s">
+      <c r="C2" s="11"/>
+      <c r="E2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="8"/>
-      <c r="H2" s="7" t="s">
+      <c r="F2" s="11"/>
+      <c r="H2" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="8"/>
-      <c r="K2" s="7" t="s">
+      <c r="I2" s="11"/>
+      <c r="K2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="L2" s="8"/>
-      <c r="N2" s="7" t="s">
+      <c r="L2" s="11"/>
+      <c r="N2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="O2" s="8"/>
-      <c r="Q2" s="7" t="s">
+      <c r="O2" s="11"/>
+      <c r="Q2" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="R2" s="8"/>
-    </row>
-    <row r="3" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="R2" s="11"/>
+    </row>
+    <row r="3" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
@@ -728,7 +755,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="2:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:18" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B4" s="4" t="s">
         <v>8</v>
       </c>
@@ -766,527 +793,554 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="2:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:18" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
-        <v>18</v>
+        <v>77</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="I5" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="9"/>
+      <c r="H5" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
       <c r="N5" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O5" s="4" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" spans="2:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="3" t="s">
-        <v>20</v>
+      <c r="Q5" s="9"/>
+      <c r="R5" s="9"/>
+    </row>
+    <row r="6" spans="2:18" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B6" s="4" t="s">
+        <v>78</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
+      <c r="H6" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>9</v>
+      </c>
       <c r="K6" s="6"/>
       <c r="L6" s="6"/>
       <c r="N6" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="O6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="R6" s="5"/>
-    </row>
-    <row r="7" spans="2:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>13</v>
+    </row>
+    <row r="7" spans="2:18" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
       <c r="K7" s="6"/>
       <c r="L7" s="6"/>
-    </row>
-    <row r="8" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B8" s="3" t="s">
+      <c r="R7" s="5"/>
+    </row>
+    <row r="8" spans="2:18" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B8" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="K8" s="6"/>
+      <c r="L8" s="6"/>
+    </row>
+    <row r="9" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="B9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="2:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="B13" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C13" s="11"/>
+      <c r="E13" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F13" s="11"/>
+      <c r="H13" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="I13" s="11"/>
+    </row>
+    <row r="14" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="B14" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="B15" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="10" spans="2:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B12" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="8"/>
-      <c r="E12" s="7" t="s">
+      <c r="E15" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I15" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F12" s="8"/>
-      <c r="H12" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="I12" s="8"/>
-    </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B13" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B14" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="H14" s="4" t="s">
+    </row>
+    <row r="16" spans="2:18" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="I14" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="2:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" s="4" t="s">
+      <c r="C16" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E15" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B16" s="3" t="s">
+      <c r="E16" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>33</v>
-      </c>
       <c r="F16" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="I16" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B17" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>9</v>
+      </c>
       <c r="E17" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="18" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
       <c r="E18" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>25</v>
       </c>
       <c r="H18" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E19" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B23" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I18" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B22" s="7" t="s">
+      <c r="C23" s="11"/>
+      <c r="E23" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C22" s="8"/>
-      <c r="E22" s="7" t="s">
+      <c r="F23" s="11"/>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B24" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B25" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="F22" s="8"/>
-    </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B23" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B24" s="3" t="s">
+      <c r="C25" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E25" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="F25" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B26" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B27" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B28" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C28" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E24" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B25" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B26" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B27" s="3" t="s">
+      <c r="E28" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="E28" s="3" t="s">
-        <v>49</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B32" s="7" t="s">
+    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="E29" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B33" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="C33" s="11"/>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B34" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B35" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C32" s="8"/>
-    </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B33" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B34" s="4" t="s">
+      <c r="C35" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C34" s="4" t="s">
+    </row>
+    <row r="36" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="4" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="35" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="4" t="s">
+      <c r="C36" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C35" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="36" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="4" t="s">
+      <c r="C37" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B38" s="6"/>
+      <c r="C38" s="6"/>
+    </row>
+    <row r="41" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B41" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="C36" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B37" s="6"/>
-      <c r="C37" s="6"/>
-    </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B40" s="7" t="s">
+      <c r="C41" s="11"/>
+      <c r="E41" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="C40" s="8"/>
-      <c r="E40" s="7" t="s">
+      <c r="F41" s="11"/>
+    </row>
+    <row r="42" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B42" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B43" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="F40" s="8"/>
-    </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B41" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B42" s="4" t="s">
+      <c r="C43" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="44" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B44" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C42" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E42" s="3" t="s">
+      <c r="C44" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="45" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B45" s="4" t="s">
         <v>58</v>
-      </c>
-      <c r="F42" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B43" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E43" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="F43" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B44" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E44" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="F44" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="45" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="4" t="s">
-        <v>62</v>
       </c>
       <c r="C45" s="4" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="46" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E45" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F45" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="46" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B46" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="F46" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="47" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B47" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E47" s="8"/>
+    </row>
+    <row r="48" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B48" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="49" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B49" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="50" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B50" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C46" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B47" s="4" t="s">
+      <c r="C50" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="51" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B51" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C47" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B48" s="4" t="s">
+      <c r="C51" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="52" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B52" s="5"/>
+    </row>
+    <row r="53" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B53" s="5"/>
+    </row>
+    <row r="55" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B55" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="C48" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="49" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B49" s="4" t="s">
+      <c r="C55" s="11"/>
+      <c r="E55" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="C49" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="50" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B50" s="4" t="s">
+      <c r="F55" s="11"/>
+    </row>
+    <row r="56" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B56" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="57" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B57" s="3" t="s">
         <v>67</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="51" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B51" s="5"/>
-    </row>
-    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B52" s="5"/>
-    </row>
-    <row r="54" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B54" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="C54" s="8"/>
-      <c r="E54" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="F54" s="8"/>
-    </row>
-    <row r="55" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B55" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="56" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B56" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C56" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E56" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="F56" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="57" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B57" s="4" t="s">
-        <v>76</v>
       </c>
       <c r="C57" s="4" t="s">
         <v>11</v>
       </c>
       <c r="E57" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F57" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="58" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B58" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="F57" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="58" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B58" s="10"/>
-      <c r="C58" s="10"/>
+      <c r="C58" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="E58" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="F58" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F58" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="G58" s="6"/>
-    </row>
-    <row r="59" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B59" s="10"/>
-      <c r="C59" s="10"/>
-      <c r="E59" s="10"/>
-      <c r="F59" s="10"/>
+    </row>
+    <row r="59" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B59" s="8"/>
+      <c r="C59" s="8"/>
+      <c r="E59" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G59" s="6"/>
+    </row>
+    <row r="60" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B60" s="8"/>
+      <c r="C60" s="8"/>
+      <c r="E60" s="8"/>
+      <c r="F60" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="E54:F54"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="E55:F55"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="Q2:R2"/>
+    <mergeCell ref="N2:O2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="H13:I13"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="H2:I2"/>
-    <mergeCell ref="Q2:R2"/>
-    <mergeCell ref="N2:O2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>